<commit_message>
test: wire the OLAP slicer and timeline fixture the way Excel does
Excel removed the slicer and timeline from the spec-derived fixture. An
Excel-saved workbook with OLAP slicers and Excel's own repairs show the
real wiring: slicers point at a dedicated slicer-data pivot cache listed
under the x14 pivotCaches extension, and a timeline points at the pivot
cache itself, which then moves to the x15 timelineCachePivotCaches list.

Claude-Session: https://claude.ai/code/session_019f7ZskFy3FHdvUjv8uKTPk
</commit_message>
<xml_diff>
--- a/crates/ripbi-core/tests/fixtures/xlsx/olap-pivots-spec-slicers-xmla.xlsx
+++ b/crates/ripbi-core/tests/fixtures/xlsx/olap-pivots-spec-slicers-xmla.xlsx
@@ -17,15 +17,27 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId3"/>
     <pivotCache cacheId="2" r:id="rId4"/>
     <pivotCache cacheId="3" r:id="rId15"/>
   </pivotCaches>
   <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{876F7934-8845-4945-9796-88D515C7AA90}">
+      <x14:pivotCaches>
+        <pivotCache cacheId="4" r:id="rId16"/>
+      </x14:pivotCaches>
+    </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
       <x14:slicerCaches>
         <x14:slicerCache r:id="rId11"/>
       </x14:slicerCaches>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
+      <x14:workbookPr/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{A2CB5862-8E78-49c6-8D9D-AF26E26ADB89}">
+      <x15:timelineCachePivotCaches>
+        <pivotCache cacheId="1" r:id="rId3"/>
+      </x15:timelineCachePivotCaches>
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}">
       <x15:timelineCacheRefs>
@@ -193,21 +205,21 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>5</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>1</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>8</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>9</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:to>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="2" name="Country"/>
@@ -223,23 +235,8 @@
             </a:graphicData>
           </a:graphic>
         </xdr:graphicFrame>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback>
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>5</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>1</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>8</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>9</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:to>
+      </mc:Choice>
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="Country"/>
@@ -267,25 +264,25 @@
             </a:p>
           </xdr:txBody>
         </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:tsle="http://schemas.microsoft.com/office/drawing/2012/timeslicer" Requires="tsle">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>9</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>1</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>12</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>9</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:to>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:tsle="http://schemas.microsoft.com/office/drawing/2012/timeslicer" Requires="tsle">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="3" name="Date"/>
@@ -301,23 +298,8 @@
             </a:graphicData>
           </a:graphic>
         </xdr:graphicFrame>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback>
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>9</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>1</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>12</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>9</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:to>
+      </mc:Choice>
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="Date"/>
@@ -345,10 +327,10 @@
             </a:p>
           </xdr:txBody>
         </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Fallback>
-  </mc:AlternateContent>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -437,7 +419,10 @@
   </maps>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1" pivotCacheId="1"/>
+      <x14:pivotCacheDefinition pivotCacheId="1048576002" supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{ABF5C744-AB39-4b91-8756-CFA1BBC848D5}">
+      <x15:pivotCacheIdVersion cacheIdSupportedVersion="0" cacheIdCreatedVersion="0"/>
     </ext>
     <ext xmlns:xxpim="http://schemas.microsoft.com/office/spreadsheetml/2020/pivotNov2020" uri="{48A13866-0669-42A6-8768-4E36796AE8C3}">
       <xxpim:implicitMeasureSupport>1</xxpim:implicitMeasureSupport>
@@ -526,7 +511,7 @@
   </tupleCache>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1" pivotCacheId="2"/>
+      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
     </ext>
   </extLst>
 </pivotCacheDefinition>
@@ -607,7 +592,43 @@
   </maps>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1" pivotCacheId="3"/>
+      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" saveData="0" backgroundQuery="1" createdVersion="3" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1">
+  <cacheSource type="external" connectionId="1">
+    <extLst>
+      <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{F057638F-6D5F-4e77-A914-E7F072B9BCA8}">
+        <x14:sourceConnection name="Sales Model"/>
+      </ext>
+    </extLst>
+  </cacheSource>
+  <cacheFields count="0"/>
+  <cacheHierarchies count="12">
+    <cacheHierarchy uniqueName="[Customer].[Country]" caption="Country" attribute="1" defaultMemberUniqueName="[Customer].[Country].[All]" allUniqueName="[Customer].[Country].[All]" dimensionUniqueName="[Customer]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Customer].[Customer Key]" caption="Customer Key" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Customer].[Customer Key].[All]" allUniqueName="[Customer].[Customer Key].[All]" dimensionUniqueName="[Customer]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Customer].[Segment]" caption="Segment" attribute="1" defaultMemberUniqueName="[Customer].[Segment].[All]" allUniqueName="[Customer].[Segment].[All]" dimensionUniqueName="[Customer]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Date].[Date]" caption="Date" attribute="1" time="1" defaultMemberUniqueName="[Date].[Date].[All]" allUniqueName="[Date].[Date].[All]" dimensionUniqueName="[Date]" displayFolder="" count="0" memberValueDatatype="7" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Date].[Year]" caption="Year" attribute="1" defaultMemberUniqueName="[Date].[Year].[All]" allUniqueName="[Date].[Year].[All]" dimensionUniqueName="[Date]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Product].[Category]" caption="Category" attribute="1" defaultMemberUniqueName="[Product].[Category].[All]" allUniqueName="[Product].[Category].[All]" dimensionUniqueName="[Product]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Product].[Product Key]" caption="Product Key" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Product].[Product Key].[All]" allUniqueName="[Product].[Product Key].[All]" dimensionUniqueName="[Product]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Sales].[Amount]" caption="Amount" attribute="1" defaultMemberUniqueName="[Sales].[Amount].[All]" allUniqueName="[Sales].[Amount].[All]" dimensionUniqueName="[Sales]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Sales].[Quantity]" caption="Quantity" attribute="1" defaultMemberUniqueName="[Sales].[Quantity].[All]" allUniqueName="[Sales].[Quantity].[All]" dimensionUniqueName="[Sales]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Total Sales]" caption="Total Sales" measure="1" displayFolder="" measureGroup="Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Order Count]" caption="Order Count" measure="1" displayFolder="Counts" measureGroup="Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Average Price]" caption="Average Price" measure="1" displayFolder="Pricing" measureGroup="Key Measures" count="0"/>
+  </cacheHierarchies>
+  <kpis count="0"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition slicerData="1" pivotCacheId="1048576001" supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
+    </ext>
+    <ext xmlns:xxpim="http://schemas.microsoft.com/office/spreadsheetml/2020/pivotNov2020" uri="{48A13866-0669-42A6-8768-4E36796AE8C3}">
+      <xxpim:implicitMeasureSupport>1</xxpim:implicitMeasureSupport>
     </ext>
   </extLst>
 </pivotCacheDefinition>
@@ -817,7 +838,7 @@
     <pivotTable tabId="3" name="Segments"/>
   </pivotTables>
   <data>
-    <olap pivotCacheId="1">
+    <olap pivotCacheId="1048576001">
       <levels count="2">
         <level uniqueName="[Customer].[Country].[(All)]" sourceCaption="(All)" count="0"/>
         <level uniqueName="[Customer].[Country].[Country]" sourceCaption="Country" count="2">
@@ -830,7 +851,7 @@
         </level>
       </levels>
       <selections count="1">
-        <selection n="[Customer].[Country].&amp;[Atlantis]"/>
+        <selection n="[Customer].[Country].[All]"/>
       </selections>
     </olap>
   </data>
@@ -848,7 +869,7 @@
   <pivotTables>
     <pivotTable tabId="2" name="Sales Model"/>
   </pivotTables>
-  <state minimalRefreshVersion="6" lastRefreshVersion="6" pivotCacheId="1" filterType="unknown">
+  <state minimalRefreshVersion="6" lastRefreshVersion="6" pivotCacheId="1048576002" filterType="unknown">
     <bounds startDate="2020-01-01T00:00:00" endDate="2021-01-01T00:00:00"/>
   </state>
 </timelineCacheDefinition>

</xml_diff>

<commit_message>
test: drop the spec-derived CUBE tuple cache from the slicer fixture
Excel repaired workbook.xml on every open until the hand-written tuple
cache behind the CUBESET formulas was removed; without it the workbook
opens cleanly. The formulas stay as text.

Claude-Session: https://claude.ai/code/session_019f7ZskFy3FHdvUjv8uKTPk
</commit_message>
<xml_diff>
--- a/crates/ripbi-core/tests/fixtures/xlsx/olap-pivots-spec-slicers-xmla.xlsx
+++ b/crates/ripbi-core/tests/fixtures/xlsx/olap-pivots-spec-slicers-xmla.xlsx
@@ -17,7 +17,6 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="2" r:id="rId4"/>
     <pivotCache cacheId="3" r:id="rId15"/>
   </pivotCaches>
   <extLst>
@@ -59,54 +58,6 @@
     <olapPr sendLocale="1" rowDrillCount="1000"/>
   </connection>
 </connections>
-</file>
-
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <metadataTypes count="1">
-    <metadataType name="XLMDX" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
-  </metadataTypes>
-  <metadataStrings count="5">
-    <s v="Sales Model"/>
-    <s v="[Product].[Category].Children"/>
-    <s v="[Measures].[Total Sales]"/>
-    <s v="[Product].[Category].&amp;[Bikes]"/>
-    <s v="#,0"/>
-  </metadataStrings>
-  <mdxMetadata count="4">
-    <mdx n="0" f="s">
-      <ms ns="1" c="1" o="d" s="2"/>
-    </mdx>
-    <mdx n="0" f="r">
-      <t c="1">
-        <n x="3"/>
-      </t>
-    </mdx>
-    <mdx n="0" f="c">
-      <ms ns="1" c="1" o="d" s="2"/>
-    </mdx>
-    <mdx n="0" f="v">
-      <t c="2" si="4">
-        <n x="2"/>
-        <n x="3"/>
-      </t>
-    </mdx>
-  </mdxMetadata>
-  <valueMetadata count="4">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-    <bk>
-      <rc t="1" v="1"/>
-    </bk>
-    <bk>
-      <rc t="1" v="2"/>
-    </bk>
-    <bk>
-      <rc t="1" v="3"/>
-    </bk>
-  </valueMetadata>
-</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -184,23 +135,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
 </styleSheet>
-</file>
-
-<file path=xl/volatileDependencies.xml><?xml version="1.0" encoding="utf-8"?>
-<volTypes xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <volType type="olapFunctions">
-    <main first="Sales Model">
-      <tp t="e">
-        <v>#N/A</v>
-        <stp>1</stp>
-        <tr r="A23" s="2"/>
-        <tr r="A22" s="2"/>
-        <tr r="A21" s="2"/>
-        <tr r="A20" s="2"/>
-      </tp>
-    </main>
-  </volType>
-</volTypes>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -431,92 +365,6 @@
 </pivotCacheDefinition>
 </file>
 
-<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" invalid="1" saveData="0" backgroundQuery="1" createdVersion="3" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" tupleCache="1" supportSubquery="1" supportAdvancedDrill="1">
-  <cacheSource type="external" connectionId="1"/>
-  <cacheFields count="2">
-    <cacheField name="[Measures].[MeasuresLevel]" caption="MeasuresLevel" numFmtId="0" hierarchy="5">
-      <sharedItems count="1">
-        <s v="[Measures].[Total Sales]" c="Total Sales"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="[Product].[Category].[Category]" caption="Category" numFmtId="0" hierarchy="6" level="1">
-      <sharedItems count="1">
-        <s v="[Product].[Category].&amp;[Bikes]" c="Bikes"/>
-      </sharedItems>
-    </cacheField>
-  </cacheFields>
-  <cacheHierarchies count="13">
-    <cacheHierarchy uniqueName="[Customer].[Country]" caption="Country" attribute="1" defaultMemberUniqueName="[Customer].[Country].[All]" allUniqueName="[Customer].[Country].[All]" allCaption="All" dimensionUniqueName="[Customer]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Customer].[Customer Key]" caption="Customer Key" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Customer].[Customer Key].[All]" allUniqueName="[Customer].[Customer Key].[All]" dimensionUniqueName="[Customer]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Customer].[Segment]" caption="Segment" attribute="1" defaultMemberUniqueName="[Customer].[Segment].[All]" allUniqueName="[Customer].[Segment].[All]" dimensionUniqueName="[Customer]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Date].[Date]" caption="Date" attribute="1" time="1" defaultMemberUniqueName="[Date].[Date].[All]" allUniqueName="[Date].[Date].[All]" dimensionUniqueName="[Date]" displayFolder="" count="0" memberValueDatatype="7" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Date].[Year]" caption="Year" attribute="1" defaultMemberUniqueName="[Date].[Year].[All]" allUniqueName="[Date].[Year].[All]" dimensionUniqueName="[Date]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Measures]" caption="Measures" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Measures].[__Default measure]" dimensionUniqueName="[Measures]" displayFolder="" measures="1" count="1" memberValueDatatype="130" unbalanced="0">
-      <fieldsUsage count="1">
-        <fieldUsage x="0"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Product].[Category]" caption="Category" attribute="1" defaultMemberUniqueName="[Product].[Category].[All]" allUniqueName="[Product].[Category].[All]" allCaption="All" dimensionUniqueName="[Product]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Product].[Product Key]" caption="Product Key" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Product].[Product Key].[All]" allUniqueName="[Product].[Product Key].[All]" dimensionUniqueName="[Product]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Sales].[Amount]" caption="Amount" attribute="1" defaultMemberUniqueName="[Sales].[Amount].[All]" allUniqueName="[Sales].[Amount].[All]" dimensionUniqueName="[Sales]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Sales].[Quantity]" caption="Quantity" attribute="1" defaultMemberUniqueName="[Sales].[Quantity].[All]" allUniqueName="[Sales].[Quantity].[All]" dimensionUniqueName="[Sales]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Total Sales]" caption="Total Sales" measure="1" displayFolder="" measureGroup="Sales" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Order Count]" caption="Order Count" measure="1" displayFolder="Counts" measureGroup="Sales" count="0"/>
-    <cacheHierarchy uniqueName="[Measures].[Average Price]" caption="Average Price" measure="1" displayFolder="Pricing" measureGroup="Key Measures" count="0"/>
-  </cacheHierarchies>
-  <kpis count="0"/>
-  <tupleCache>
-    <entries count="1">
-      <m in="0">
-        <tpls c="3">
-          <tpl fld="0" item="0"/>
-          <tpl fld="1" item="0"/>
-          <tpl hier="0" item="4294967295"/>
-        </tpls>
-      </m>
-    </entries>
-    <sets count="1">
-      <set count="1" maxRank="1" setDefinition="[Product].[Category].Children" sortType="descending">
-        <tpls c="1">
-          <tpl fld="1" item="0"/>
-        </tpls>
-        <sortByTuple c="1">
-          <tpl fld="0" item="0"/>
-        </sortByTuple>
-      </set>
-    </sets>
-    <queryCache count="5">
-      <query mdx=""/>
-      <query mdx="[Product].[Category].Children"/>
-      <query mdx="[Measures].[Total Sales]">
-        <tpls c="1">
-          <tpl fld="0" item="0"/>
-        </tpls>
-      </query>
-      <query mdx="[Customer].[Country].[All]">
-        <tpls c="1">
-          <tpl hier="0" item="4294967295"/>
-        </tpls>
-      </query>
-      <query mdx="[Product].[Category].&amp;[Bikes]">
-        <tpls c="1">
-          <tpl hier="1" item="0"/>
-        </tpls>
-      </query>
-    </queryCache>
-    <serverFormats count="1">
-      <serverFormat format="#,0"/>
-    </serverFormats>
-  </tupleCache>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
 <file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" saveData="0" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1">
   <cacheSource type="external" connectionId="2"/>
@@ -934,25 +782,25 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="str" vm="1">
+      <c r="A20" t="str">
         <f>CUBESET("Sales Model","[Product].[Category].Children","Categories",2,"[Measures].[Total Sales]")</f>
         <v>Categories</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="str" vm="2">
+      <c r="A21" t="str">
         <f>CUBERANKEDMEMBER("Sales Model",$A$20,1)</f>
         <v>Bikes</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" vm="3">
+      <c r="A22">
         <f>CUBESETCOUNT($A$20)</f>
         <v>1</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" vm="4">
+      <c r="A23" s="1">
         <f>CUBEVALUE("Sales Model","[Measures].[Total Sales]",$A$21,Slicer_Country)</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
test: restore the CUBE tuple cache in the slicer fixture, Excel-clean
Rebuilt to the shape of a real Excel tuple cache (only the MeasuresLevel
field, no sets element); Excel 365 opens the workbook without repairs.

Claude-Session: https://claude.ai/code/session_019f7ZskFy3FHdvUjv8uKTPk
</commit_message>
<xml_diff>
--- a/crates/ripbi-core/tests/fixtures/xlsx/olap-pivots-spec-slicers-xmla.xlsx
+++ b/crates/ripbi-core/tests/fixtures/xlsx/olap-pivots-spec-slicers-xmla.xlsx
@@ -17,6 +17,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
+    <pivotCache cacheId="2" r:id="rId4"/>
     <pivotCache cacheId="3" r:id="rId15"/>
   </pivotCaches>
   <extLst>
@@ -58,6 +59,54 @@
     <olapPr sendLocale="1" rowDrillCount="1000"/>
   </connection>
 </connections>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <metadataTypes count="1">
+    <metadataType name="XLMDX" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <metadataStrings count="5">
+    <s v="Sales Model"/>
+    <s v="[Product].[Category].Children"/>
+    <s v="[Measures].[Total Sales]"/>
+    <s v="[Product].[Category].&amp;[Bikes]"/>
+    <s v="#,0"/>
+  </metadataStrings>
+  <mdxMetadata count="4">
+    <mdx n="0" f="s">
+      <ms ns="1" c="1" o="d" s="2"/>
+    </mdx>
+    <mdx n="0" f="r">
+      <t c="1">
+        <n x="3"/>
+      </t>
+    </mdx>
+    <mdx n="0" f="c">
+      <ms ns="1" c="1" o="d" s="2"/>
+    </mdx>
+    <mdx n="0" f="v">
+      <t c="2" si="4">
+        <n x="2"/>
+        <n x="3"/>
+      </t>
+    </mdx>
+  </mdxMetadata>
+  <valueMetadata count="4">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+    <bk>
+      <rc t="1" v="1"/>
+    </bk>
+    <bk>
+      <rc t="1" v="2"/>
+    </bk>
+    <bk>
+      <rc t="1" v="3"/>
+    </bk>
+  </valueMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -135,6 +184,23 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
 </styleSheet>
+</file>
+
+<file path=xl/volatileDependencies.xml><?xml version="1.0" encoding="utf-8"?>
+<volTypes xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <volType type="olapFunctions">
+    <main first="Sales Model">
+      <tp t="e">
+        <v>#N/A</v>
+        <stp>1</stp>
+        <tr r="A23" s="2"/>
+        <tr r="A22" s="2"/>
+        <tr r="A21" s="2"/>
+        <tr r="A20" s="2"/>
+      </tp>
+    </main>
+  </volType>
+</volTypes>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -365,6 +431,71 @@
 </pivotCacheDefinition>
 </file>
 
+<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" invalid="1" saveData="0" backgroundQuery="1" createdVersion="3" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" tupleCache="1" supportSubquery="1" supportAdvancedDrill="1">
+  <cacheSource type="external" connectionId="1"/>
+  <cacheFields count="1">
+    <cacheField name="[Measures].[MeasuresLevel]" caption="MeasuresLevel" numFmtId="0" hierarchy="5">
+      <sharedItems count="1">
+        <s v="[Measures].[Total Sales]" c="Total Sales"/>
+      </sharedItems>
+    </cacheField>
+  </cacheFields>
+  <cacheHierarchies count="13">
+    <cacheHierarchy uniqueName="[Customer].[Country]" caption="Country" attribute="1" defaultMemberUniqueName="[Customer].[Country].[All]" allUniqueName="[Customer].[Country].[All]" allCaption="All" dimensionUniqueName="[Customer]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Customer].[Customer Key]" caption="Customer Key" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Customer].[Customer Key].[All]" allUniqueName="[Customer].[Customer Key].[All]" dimensionUniqueName="[Customer]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Customer].[Segment]" caption="Segment" attribute="1" defaultMemberUniqueName="[Customer].[Segment].[All]" allUniqueName="[Customer].[Segment].[All]" dimensionUniqueName="[Customer]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Date].[Date]" caption="Date" attribute="1" time="1" defaultMemberUniqueName="[Date].[Date].[All]" allUniqueName="[Date].[Date].[All]" dimensionUniqueName="[Date]" displayFolder="" count="0" memberValueDatatype="7" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Date].[Year]" caption="Year" attribute="1" defaultMemberUniqueName="[Date].[Year].[All]" allUniqueName="[Date].[Year].[All]" dimensionUniqueName="[Date]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Measures]" caption="Measures" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Measures].[__Default measure]" dimensionUniqueName="[Measures]" displayFolder="" measures="1" count="1" memberValueDatatype="130" unbalanced="0">
+      <fieldsUsage count="1">
+        <fieldUsage x="0"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Product].[Category]" caption="Category" attribute="1" defaultMemberUniqueName="[Product].[Category].[All]" allUniqueName="[Product].[Category].[All]" allCaption="All" dimensionUniqueName="[Product]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Product].[Product Key]" caption="Product Key" attribute="1" keyAttribute="1" defaultMemberUniqueName="[Product].[Product Key].[All]" allUniqueName="[Product].[Product Key].[All]" dimensionUniqueName="[Product]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Sales].[Amount]" caption="Amount" attribute="1" defaultMemberUniqueName="[Sales].[Amount].[All]" allUniqueName="[Sales].[Amount].[All]" dimensionUniqueName="[Sales]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Sales].[Quantity]" caption="Quantity" attribute="1" defaultMemberUniqueName="[Sales].[Quantity].[All]" allUniqueName="[Sales].[Quantity].[All]" dimensionUniqueName="[Sales]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Total Sales]" caption="Total Sales" measure="1" displayFolder="" measureGroup="Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Order Count]" caption="Order Count" measure="1" displayFolder="Counts" measureGroup="Sales" count="0"/>
+    <cacheHierarchy uniqueName="[Measures].[Average Price]" caption="Average Price" measure="1" displayFolder="Pricing" measureGroup="Key Measures" count="0"/>
+  </cacheHierarchies>
+  <kpis count="0"/>
+  <tupleCache>
+    <entries count="1">
+      <m in="0">
+        <tpls c="2">
+          <tpl hier="0" item="4294967295"/>
+          <tpl fld="0" item="0"/>
+        </tpls>
+      </m>
+    </entries>
+    <queryCache count="4">
+      <query mdx=""/>
+      <query mdx="[Product].[Category].Children"/>
+      <query mdx="[Measures].[Total Sales]">
+        <tpls c="1">
+          <tpl fld="0" item="0"/>
+        </tpls>
+      </query>
+      <query mdx="[Customer].[Country].[All]">
+        <tpls c="1">
+          <tpl hier="0" item="4294967295"/>
+        </tpls>
+      </query>
+    </queryCache>
+    <serverFormats count="1">
+      <serverFormat format="#,0"/>
+    </serverFormats>
+  </tupleCache>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
 <file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" saveData="0" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1">
   <cacheSource type="external" connectionId="2"/>
@@ -782,25 +913,25 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="str">
+      <c r="A20" t="str" vm="1">
         <f>CUBESET("Sales Model","[Product].[Category].Children","Categories",2,"[Measures].[Total Sales]")</f>
         <v>Categories</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="str">
+      <c r="A21" t="str" vm="2">
         <f>CUBERANKEDMEMBER("Sales Model",$A$20,1)</f>
         <v>Bikes</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22">
+      <c r="A22" vm="3">
         <f>CUBESETCOUNT($A$20)</f>
         <v>1</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1">
+      <c r="A23" s="1" vm="4">
         <f>CUBEVALUE("Sales Model","[Measures].[Total Sales]",$A$21,Slicer_Country)</f>
         <v>0</v>
       </c>

</xml_diff>